<commit_message>
Leave policy fixed shipment cost blank to inherit from Mode
SCG rejects the vehicle cost name in TG_Policies.Fixed Shipment Cost.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QzcZa6LEpCqhNBeutDq5dQ
</commit_message>
<xml_diff>
--- a/ms6_BatchExport_input_corregido.xlsx
+++ b/ms6_BatchExport_input_corregido.xlsx
@@ -3173,11 +3173,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T2" t="inlineStr">
         <is>
           <t>950</t>
@@ -3212,7 +3207,7 @@
       </c>
       <c r="BL2" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM2" t="inlineStr">
@@ -3285,11 +3280,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T3" t="inlineStr">
         <is>
           <t>950</t>
@@ -3324,7 +3314,7 @@
       </c>
       <c r="BL3" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM3" t="inlineStr">
@@ -3397,11 +3387,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
           <t>950</t>
@@ -3436,7 +3421,7 @@
       </c>
       <c r="BL4" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM4" t="inlineStr">
@@ -3509,11 +3494,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T5" t="inlineStr">
         <is>
           <t>950</t>
@@ -3548,7 +3528,7 @@
       </c>
       <c r="BL5" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM5" t="inlineStr">
@@ -3621,11 +3601,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T6" t="inlineStr">
         <is>
           <t>950</t>
@@ -3660,7 +3635,7 @@
       </c>
       <c r="BL6" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM6" t="inlineStr">
@@ -3733,11 +3708,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T7" t="inlineStr">
         <is>
           <t>950</t>
@@ -3772,7 +3742,7 @@
       </c>
       <c r="BL7" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM7" t="inlineStr">
@@ -3845,11 +3815,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T8" t="inlineStr">
         <is>
           <t>950</t>
@@ -3884,7 +3849,7 @@
       </c>
       <c r="BL8" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM8" t="inlineStr">
@@ -3957,11 +3922,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T9" t="inlineStr">
         <is>
           <t>950</t>
@@ -3996,7 +3956,7 @@
       </c>
       <c r="BL9" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM9" t="inlineStr">
@@ -4069,11 +4029,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T10" t="inlineStr">
         <is>
           <t>950</t>
@@ -4108,7 +4063,7 @@
       </c>
       <c r="BL10" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM10" t="inlineStr">
@@ -4181,11 +4136,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T11" t="inlineStr">
         <is>
           <t>950</t>
@@ -4220,7 +4170,7 @@
       </c>
       <c r="BL11" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM11" t="inlineStr">
@@ -4293,11 +4243,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T12" t="inlineStr">
         <is>
           <t>950</t>
@@ -4332,7 +4277,7 @@
       </c>
       <c r="BL12" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM12" t="inlineStr">
@@ -4405,11 +4350,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T13" t="inlineStr">
         <is>
           <t>950</t>
@@ -4444,7 +4384,7 @@
       </c>
       <c r="BL13" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM13" t="inlineStr">
@@ -4517,11 +4457,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T14" t="inlineStr">
         <is>
           <t>950</t>
@@ -4556,7 +4491,7 @@
       </c>
       <c r="BL14" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM14" t="inlineStr">
@@ -4629,11 +4564,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T15" t="inlineStr">
         <is>
           <t>950</t>
@@ -4668,7 +4598,7 @@
       </c>
       <c r="BL15" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM15" t="inlineStr">
@@ -4741,11 +4671,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T16" t="inlineStr">
         <is>
           <t>950</t>
@@ -4780,7 +4705,7 @@
       </c>
       <c r="BL16" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM16" t="inlineStr">
@@ -4853,11 +4778,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T17" t="inlineStr">
         <is>
           <t>950</t>
@@ -4892,7 +4812,7 @@
       </c>
       <c r="BL17" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM17" t="inlineStr">
@@ -4965,11 +4885,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T18" t="inlineStr">
         <is>
           <t>950</t>
@@ -5004,7 +4919,7 @@
       </c>
       <c r="BL18" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM18" t="inlineStr">
@@ -5077,11 +4992,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T19" t="inlineStr">
         <is>
           <t>950</t>
@@ -5116,7 +5026,7 @@
       </c>
       <c r="BL19" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM19" t="inlineStr">
@@ -5189,11 +5099,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T20" t="inlineStr">
         <is>
           <t>950</t>
@@ -5228,7 +5133,7 @@
       </c>
       <c r="BL20" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM20" t="inlineStr">
@@ -5301,11 +5206,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T21" t="inlineStr">
         <is>
           <t>950</t>
@@ -5340,7 +5240,7 @@
       </c>
       <c r="BL21" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM21" t="inlineStr">
@@ -5413,11 +5313,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T22" t="inlineStr">
         <is>
           <t>950</t>
@@ -5452,7 +5347,7 @@
       </c>
       <c r="BL22" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM22" t="inlineStr">
@@ -5525,11 +5420,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T23" t="inlineStr">
         <is>
           <t>950</t>
@@ -5564,7 +5454,7 @@
       </c>
       <c r="BL23" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM23" t="inlineStr">
@@ -5637,11 +5527,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T24" t="inlineStr">
         <is>
           <t>950</t>
@@ -5676,7 +5561,7 @@
       </c>
       <c r="BL24" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM24" t="inlineStr">
@@ -5749,11 +5634,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T25" t="inlineStr">
         <is>
           <t>950</t>
@@ -5788,7 +5668,7 @@
       </c>
       <c r="BL25" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM25" t="inlineStr">
@@ -5861,11 +5741,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T26" t="inlineStr">
         <is>
           <t>950</t>
@@ -5900,7 +5775,7 @@
       </c>
       <c r="BL26" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM26" t="inlineStr">
@@ -5973,11 +5848,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T27" t="inlineStr">
         <is>
           <t>950</t>
@@ -6012,7 +5882,7 @@
       </c>
       <c r="BL27" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM27" t="inlineStr">
@@ -6085,11 +5955,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T28" t="inlineStr">
         <is>
           <t>950</t>
@@ -6124,7 +5989,7 @@
       </c>
       <c r="BL28" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM28" t="inlineStr">
@@ -6197,11 +6062,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T29" t="inlineStr">
         <is>
           <t>950</t>
@@ -6236,7 +6096,7 @@
       </c>
       <c r="BL29" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM29" t="inlineStr">
@@ -6309,11 +6169,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T30" t="inlineStr">
         <is>
           <t>950</t>
@@ -6348,7 +6203,7 @@
       </c>
       <c r="BL30" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM30" t="inlineStr">
@@ -6421,11 +6276,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T31" t="inlineStr">
         <is>
           <t>950</t>
@@ -6460,7 +6310,7 @@
       </c>
       <c r="BL31" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM31" t="inlineStr">
@@ -6533,11 +6383,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T32" t="inlineStr">
         <is>
           <t>950</t>
@@ -6572,7 +6417,7 @@
       </c>
       <c r="BL32" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM32" t="inlineStr">
@@ -6645,11 +6490,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T33" t="inlineStr">
         <is>
           <t>950</t>
@@ -6684,7 +6524,7 @@
       </c>
       <c r="BL33" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM33" t="inlineStr">
@@ -6757,11 +6597,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T34" t="inlineStr">
         <is>
           <t>950</t>
@@ -6796,7 +6631,7 @@
       </c>
       <c r="BL34" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM34" t="inlineStr">
@@ -6869,11 +6704,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T35" t="inlineStr">
         <is>
           <t>950</t>
@@ -6908,7 +6738,7 @@
       </c>
       <c r="BL35" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM35" t="inlineStr">
@@ -6981,11 +6811,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T36" t="inlineStr">
         <is>
           <t>950</t>
@@ -7020,7 +6845,7 @@
       </c>
       <c r="BL36" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM36" t="inlineStr">
@@ -7093,11 +6918,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T37" t="inlineStr">
         <is>
           <t>950</t>
@@ -7132,7 +6952,7 @@
       </c>
       <c r="BL37" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM37" t="inlineStr">
@@ -7205,11 +7025,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T38" t="inlineStr">
         <is>
           <t>950</t>
@@ -7244,7 +7059,7 @@
       </c>
       <c r="BL38" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM38" t="inlineStr">
@@ -7317,11 +7132,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T39" t="inlineStr">
         <is>
           <t>950</t>
@@ -7356,7 +7166,7 @@
       </c>
       <c r="BL39" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM39" t="inlineStr">
@@ -7429,11 +7239,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T40" t="inlineStr">
         <is>
           <t>950</t>
@@ -7468,7 +7273,7 @@
       </c>
       <c r="BL40" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM40" t="inlineStr">
@@ -7541,11 +7346,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T41" t="inlineStr">
         <is>
           <t>950</t>
@@ -7580,7 +7380,7 @@
       </c>
       <c r="BL41" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM41" t="inlineStr">
@@ -7653,11 +7453,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T42" t="inlineStr">
         <is>
           <t>950</t>
@@ -7692,7 +7487,7 @@
       </c>
       <c r="BL42" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM42" t="inlineStr">
@@ -7765,11 +7560,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T43" t="inlineStr">
         <is>
           <t>950</t>
@@ -7804,7 +7594,7 @@
       </c>
       <c r="BL43" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM43" t="inlineStr">
@@ -7877,11 +7667,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T44" t="inlineStr">
         <is>
           <t>950</t>
@@ -7916,7 +7701,7 @@
       </c>
       <c r="BL44" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM44" t="inlineStr">
@@ -7989,11 +7774,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T45" t="inlineStr">
         <is>
           <t>950</t>
@@ -8028,7 +7808,7 @@
       </c>
       <c r="BL45" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM45" t="inlineStr">
@@ -8101,11 +7881,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T46" t="inlineStr">
         <is>
           <t>950</t>
@@ -8140,7 +7915,7 @@
       </c>
       <c r="BL46" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM46" t="inlineStr">
@@ -8213,11 +7988,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T47" t="inlineStr">
         <is>
           <t>950</t>
@@ -8252,7 +8022,7 @@
       </c>
       <c r="BL47" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM47" t="inlineStr">
@@ -8325,11 +8095,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T48" t="inlineStr">
         <is>
           <t>950</t>
@@ -8364,7 +8129,7 @@
       </c>
       <c r="BL48" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM48" t="inlineStr">
@@ -8437,11 +8202,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T49" t="inlineStr">
         <is>
           <t>950</t>
@@ -8476,7 +8236,7 @@
       </c>
       <c r="BL49" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM49" t="inlineStr">
@@ -8549,11 +8309,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T50" t="inlineStr">
         <is>
           <t>950</t>
@@ -8588,7 +8343,7 @@
       </c>
       <c r="BL50" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM50" t="inlineStr">
@@ -8661,11 +8416,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T51" t="inlineStr">
         <is>
           <t>950</t>
@@ -8700,7 +8450,7 @@
       </c>
       <c r="BL51" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM51" t="inlineStr">
@@ -8773,11 +8523,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T52" t="inlineStr">
         <is>
           <t>950</t>
@@ -8812,7 +8557,7 @@
       </c>
       <c r="BL52" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM52" t="inlineStr">
@@ -8885,11 +8630,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S53" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T53" t="inlineStr">
         <is>
           <t>950</t>
@@ -8924,7 +8664,7 @@
       </c>
       <c r="BL53" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM53" t="inlineStr">
@@ -8997,11 +8737,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S54" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T54" t="inlineStr">
         <is>
           <t>950</t>
@@ -9036,7 +8771,7 @@
       </c>
       <c r="BL54" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM54" t="inlineStr">
@@ -9109,11 +8844,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T55" t="inlineStr">
         <is>
           <t>950</t>
@@ -9148,7 +8878,7 @@
       </c>
       <c r="BL55" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM55" t="inlineStr">
@@ -9221,11 +8951,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T56" t="inlineStr">
         <is>
           <t>950</t>
@@ -9260,7 +8985,7 @@
       </c>
       <c r="BL56" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM56" t="inlineStr">
@@ -9333,11 +9058,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T57" t="inlineStr">
         <is>
           <t>950</t>
@@ -9372,7 +9092,7 @@
       </c>
       <c r="BL57" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM57" t="inlineStr">
@@ -9445,11 +9165,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T58" t="inlineStr">
         <is>
           <t>950</t>
@@ -9484,7 +9199,7 @@
       </c>
       <c r="BL58" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM58" t="inlineStr">
@@ -9557,11 +9272,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S59" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T59" t="inlineStr">
         <is>
           <t>950</t>
@@ -9596,7 +9306,7 @@
       </c>
       <c r="BL59" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM59" t="inlineStr">
@@ -9669,11 +9379,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S60" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T60" t="inlineStr">
         <is>
           <t>950</t>
@@ -9708,7 +9413,7 @@
       </c>
       <c r="BL60" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM60" t="inlineStr">
@@ -9781,11 +9486,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S61" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T61" t="inlineStr">
         <is>
           <t>950</t>
@@ -9820,7 +9520,7 @@
       </c>
       <c r="BL61" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM61" t="inlineStr">
@@ -9893,11 +9593,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T62" t="inlineStr">
         <is>
           <t>950</t>
@@ -9932,7 +9627,7 @@
       </c>
       <c r="BL62" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM62" t="inlineStr">
@@ -10005,11 +9700,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S63" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T63" t="inlineStr">
         <is>
           <t>950</t>
@@ -10044,7 +9734,7 @@
       </c>
       <c r="BL63" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM63" t="inlineStr">
@@ -10117,11 +9807,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S64" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T64" t="inlineStr">
         <is>
           <t>950</t>
@@ -10156,7 +9841,7 @@
       </c>
       <c r="BL64" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM64" t="inlineStr">
@@ -10229,11 +9914,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S65" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T65" t="inlineStr">
         <is>
           <t>950</t>
@@ -10268,7 +9948,7 @@
       </c>
       <c r="BL65" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM65" t="inlineStr">
@@ -10341,11 +10021,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S66" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T66" t="inlineStr">
         <is>
           <t>950</t>
@@ -10380,7 +10055,7 @@
       </c>
       <c r="BL66" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM66" t="inlineStr">
@@ -10453,11 +10128,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S67" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T67" t="inlineStr">
         <is>
           <t>950</t>
@@ -10492,7 +10162,7 @@
       </c>
       <c r="BL67" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM67" t="inlineStr">
@@ -10565,11 +10235,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S68" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T68" t="inlineStr">
         <is>
           <t>950</t>
@@ -10604,7 +10269,7 @@
       </c>
       <c r="BL68" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM68" t="inlineStr">
@@ -10677,11 +10342,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S69" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T69" t="inlineStr">
         <is>
           <t>950</t>
@@ -10716,7 +10376,7 @@
       </c>
       <c r="BL69" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM69" t="inlineStr">
@@ -10789,11 +10449,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S70" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T70" t="inlineStr">
         <is>
           <t>950</t>
@@ -10828,7 +10483,7 @@
       </c>
       <c r="BL70" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM70" t="inlineStr">
@@ -10901,11 +10556,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S71" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T71" t="inlineStr">
         <is>
           <t>950</t>
@@ -10940,7 +10590,7 @@
       </c>
       <c r="BL71" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM71" t="inlineStr">
@@ -11013,11 +10663,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S72" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T72" t="inlineStr">
         <is>
           <t>950</t>
@@ -11052,7 +10697,7 @@
       </c>
       <c r="BL72" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM72" t="inlineStr">
@@ -11125,11 +10770,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S73" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T73" t="inlineStr">
         <is>
           <t>950</t>
@@ -11164,7 +10804,7 @@
       </c>
       <c r="BL73" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM73" t="inlineStr">
@@ -11237,11 +10877,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S74" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T74" t="inlineStr">
         <is>
           <t>950</t>
@@ -11276,7 +10911,7 @@
       </c>
       <c r="BL74" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM74" t="inlineStr">
@@ -11349,11 +10984,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S75" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T75" t="inlineStr">
         <is>
           <t>950</t>
@@ -11388,7 +11018,7 @@
       </c>
       <c r="BL75" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM75" t="inlineStr">
@@ -11461,11 +11091,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S76" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T76" t="inlineStr">
         <is>
           <t>950</t>
@@ -11500,7 +11125,7 @@
       </c>
       <c r="BL76" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM76" t="inlineStr">
@@ -11573,11 +11198,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S77" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T77" t="inlineStr">
         <is>
           <t>950</t>
@@ -11612,7 +11232,7 @@
       </c>
       <c r="BL77" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM77" t="inlineStr">
@@ -11685,11 +11305,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S78" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T78" t="inlineStr">
         <is>
           <t>950</t>
@@ -11724,7 +11339,7 @@
       </c>
       <c r="BL78" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM78" t="inlineStr">
@@ -11797,11 +11412,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S79" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T79" t="inlineStr">
         <is>
           <t>950</t>
@@ -11836,7 +11446,7 @@
       </c>
       <c r="BL79" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM79" t="inlineStr">
@@ -11909,11 +11519,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S80" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T80" t="inlineStr">
         <is>
           <t>950</t>
@@ -11948,7 +11553,7 @@
       </c>
       <c r="BL80" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM80" t="inlineStr">
@@ -12021,11 +11626,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S81" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T81" t="inlineStr">
         <is>
           <t>950</t>
@@ -12060,7 +11660,7 @@
       </c>
       <c r="BL81" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM81" t="inlineStr">
@@ -12133,11 +11733,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S82" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T82" t="inlineStr">
         <is>
           <t>950</t>
@@ -12172,7 +11767,7 @@
       </c>
       <c r="BL82" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM82" t="inlineStr">
@@ -12245,11 +11840,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S83" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T83" t="inlineStr">
         <is>
           <t>950</t>
@@ -12284,7 +11874,7 @@
       </c>
       <c r="BL83" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM83" t="inlineStr">
@@ -12357,11 +11947,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S84" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T84" t="inlineStr">
         <is>
           <t>950</t>
@@ -12396,7 +11981,7 @@
       </c>
       <c r="BL84" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM84" t="inlineStr">
@@ -12469,11 +12054,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S85" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T85" t="inlineStr">
         <is>
           <t>950</t>
@@ -12508,7 +12088,7 @@
       </c>
       <c r="BL85" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM85" t="inlineStr">
@@ -12581,11 +12161,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S86" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T86" t="inlineStr">
         <is>
           <t>950</t>
@@ -12620,7 +12195,7 @@
       </c>
       <c r="BL86" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM86" t="inlineStr">
@@ -12693,11 +12268,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S87" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T87" t="inlineStr">
         <is>
           <t>950</t>
@@ -12732,7 +12302,7 @@
       </c>
       <c r="BL87" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM87" t="inlineStr">
@@ -12805,11 +12375,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S88" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T88" t="inlineStr">
         <is>
           <t>950</t>
@@ -12844,7 +12409,7 @@
       </c>
       <c r="BL88" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM88" t="inlineStr">
@@ -12917,11 +12482,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S89" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T89" t="inlineStr">
         <is>
           <t>950</t>
@@ -12956,7 +12516,7 @@
       </c>
       <c r="BL89" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM89" t="inlineStr">
@@ -13029,11 +12589,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S90" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T90" t="inlineStr">
         <is>
           <t>950</t>
@@ -13068,7 +12623,7 @@
       </c>
       <c r="BL90" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM90" t="inlineStr">
@@ -13141,11 +12696,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S91" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T91" t="inlineStr">
         <is>
           <t>950</t>
@@ -13180,7 +12730,7 @@
       </c>
       <c r="BL91" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM91" t="inlineStr">
@@ -13253,11 +12803,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S92" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T92" t="inlineStr">
         <is>
           <t>950</t>
@@ -13292,7 +12837,7 @@
       </c>
       <c r="BL92" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM92" t="inlineStr">
@@ -13365,11 +12910,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S93" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T93" t="inlineStr">
         <is>
           <t>950</t>
@@ -13404,7 +12944,7 @@
       </c>
       <c r="BL93" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM93" t="inlineStr">
@@ -13477,11 +13017,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S94" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T94" t="inlineStr">
         <is>
           <t>950</t>
@@ -13516,7 +13051,7 @@
       </c>
       <c r="BL94" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM94" t="inlineStr">
@@ -13589,11 +13124,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S95" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T95" t="inlineStr">
         <is>
           <t>950</t>
@@ -13628,7 +13158,7 @@
       </c>
       <c r="BL95" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM95" t="inlineStr">
@@ -13701,11 +13231,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S96" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T96" t="inlineStr">
         <is>
           <t>950</t>
@@ -13740,7 +13265,7 @@
       </c>
       <c r="BL96" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM96" t="inlineStr">
@@ -13813,11 +13338,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S97" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T97" t="inlineStr">
         <is>
           <t>950</t>
@@ -13852,7 +13372,7 @@
       </c>
       <c r="BL97" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM97" t="inlineStr">
@@ -13925,11 +13445,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S98" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T98" t="inlineStr">
         <is>
           <t>950</t>
@@ -13964,7 +13479,7 @@
       </c>
       <c r="BL98" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM98" t="inlineStr">
@@ -14037,11 +13552,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S99" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T99" t="inlineStr">
         <is>
           <t>950</t>
@@ -14076,7 +13586,7 @@
       </c>
       <c r="BL99" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM99" t="inlineStr">
@@ -14149,11 +13659,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S100" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T100" t="inlineStr">
         <is>
           <t>950</t>
@@ -14188,7 +13693,7 @@
       </c>
       <c r="BL100" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM100" t="inlineStr">
@@ -14261,11 +13766,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S101" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T101" t="inlineStr">
         <is>
           <t>950</t>
@@ -14300,7 +13800,7 @@
       </c>
       <c r="BL101" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM101" t="inlineStr">
@@ -14373,11 +13873,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S102" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T102" t="inlineStr">
         <is>
           <t>950</t>
@@ -14412,7 +13907,7 @@
       </c>
       <c r="BL102" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM102" t="inlineStr">
@@ -14485,11 +13980,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S103" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T103" t="inlineStr">
         <is>
           <t>950</t>
@@ -14524,7 +14014,7 @@
       </c>
       <c r="BL103" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM103" t="inlineStr">
@@ -14597,11 +14087,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S104" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T104" t="inlineStr">
         <is>
           <t>950</t>
@@ -14636,7 +14121,7 @@
       </c>
       <c r="BL104" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM104" t="inlineStr">
@@ -14709,11 +14194,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S105" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T105" t="inlineStr">
         <is>
           <t>950</t>
@@ -14748,7 +14228,7 @@
       </c>
       <c r="BL105" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM105" t="inlineStr">
@@ -14821,11 +14301,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S106" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T106" t="inlineStr">
         <is>
           <t>950</t>
@@ -14860,7 +14335,7 @@
       </c>
       <c r="BL106" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM106" t="inlineStr">
@@ -14933,11 +14408,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S107" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T107" t="inlineStr">
         <is>
           <t>950</t>
@@ -14972,7 +14442,7 @@
       </c>
       <c r="BL107" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM107" t="inlineStr">
@@ -15045,11 +14515,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S108" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T108" t="inlineStr">
         <is>
           <t>950</t>
@@ -15084,7 +14549,7 @@
       </c>
       <c r="BL108" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM108" t="inlineStr">
@@ -15157,11 +14622,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S109" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T109" t="inlineStr">
         <is>
           <t>950</t>
@@ -15196,7 +14656,7 @@
       </c>
       <c r="BL109" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM109" t="inlineStr">
@@ -15269,11 +14729,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S110" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T110" t="inlineStr">
         <is>
           <t>950</t>
@@ -15308,7 +14763,7 @@
       </c>
       <c r="BL110" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM110" t="inlineStr">
@@ -15381,11 +14836,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S111" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T111" t="inlineStr">
         <is>
           <t>950</t>
@@ -15420,7 +14870,7 @@
       </c>
       <c r="BL111" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM111" t="inlineStr">
@@ -15493,11 +14943,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S112" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T112" t="inlineStr">
         <is>
           <t>950</t>
@@ -15532,7 +14977,7 @@
       </c>
       <c r="BL112" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM112" t="inlineStr">
@@ -15605,11 +15050,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S113" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T113" t="inlineStr">
         <is>
           <t>950</t>
@@ -15644,7 +15084,7 @@
       </c>
       <c r="BL113" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM113" t="inlineStr">
@@ -15717,11 +15157,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S114" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T114" t="inlineStr">
         <is>
           <t>950</t>
@@ -15756,7 +15191,7 @@
       </c>
       <c r="BL114" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM114" t="inlineStr">
@@ -15829,11 +15264,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S115" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T115" t="inlineStr">
         <is>
           <t>950</t>
@@ -15868,7 +15298,7 @@
       </c>
       <c r="BL115" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM115" t="inlineStr">
@@ -15941,11 +15371,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S116" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T116" t="inlineStr">
         <is>
           <t>950</t>
@@ -15980,7 +15405,7 @@
       </c>
       <c r="BL116" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM116" t="inlineStr">
@@ -16053,11 +15478,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S117" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T117" t="inlineStr">
         <is>
           <t>950</t>
@@ -16092,7 +15512,7 @@
       </c>
       <c r="BL117" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM117" t="inlineStr">
@@ -16165,11 +15585,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S118" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T118" t="inlineStr">
         <is>
           <t>950</t>
@@ -16204,7 +15619,7 @@
       </c>
       <c r="BL118" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM118" t="inlineStr">
@@ -16277,11 +15692,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S119" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T119" t="inlineStr">
         <is>
           <t>950</t>
@@ -16316,7 +15726,7 @@
       </c>
       <c r="BL119" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM119" t="inlineStr">
@@ -16389,11 +15799,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S120" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T120" t="inlineStr">
         <is>
           <t>950</t>
@@ -16428,7 +15833,7 @@
       </c>
       <c r="BL120" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM120" t="inlineStr">
@@ -16501,11 +15906,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S121" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T121" t="inlineStr">
         <is>
           <t>950</t>
@@ -16540,7 +15940,7 @@
       </c>
       <c r="BL121" t="inlineStr">
         <is>
-          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Linea recta (haversine) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM121" t="inlineStr">
@@ -16613,11 +16013,6 @@
           <t>Quantity-Distance</t>
         </is>
       </c>
-      <c r="S122" t="inlineStr">
-        <is>
-          <t>Camion GDL PseudoRouting</t>
-        </is>
-      </c>
       <c r="T122" t="inlineStr">
         <is>
           <t>950</t>
@@ -16652,7 +16047,7 @@
       </c>
       <c r="BL122" t="inlineStr">
         <is>
-          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX: Fixed Shipment Cost = nombre del Vehicle Cost (antes 0 anulaba al Mode); Variable vacio para no pisar la estimacion.</t>
+          <t>Distancia REAL (Bing) -- Fixed/Variable en 0 A PROPOSITO: el costo de este Mode debe calcularlo el Multi-Stop Estimation (PseudoRouting), no una tarifa fija precargada | FIX v2: Fixed Shipment Cost vacio para heredar del Mode (la politica no acepta el nombre del Vehicle Cost).</t>
         </is>
       </c>
       <c r="BM122" t="inlineStr">

</xml_diff>